<commit_message>
Dashboard de Reportes 100% funcional
</commit_message>
<xml_diff>
--- a/2026_07_06.xlsx
+++ b/2026_07_06.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -814,6 +814,126 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Juan Emilio Perez Ramirez</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>04:20:47 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Juan Emilio Perez Ramirez</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>04:29:11 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Juan Emilio Perez Ramirez</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>05:37:37 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Juan Emilio Perez Ramirez</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>05:37:58 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Juan Emilio Perez Ramirez</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>05:42:32 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Juan Emilio Perez Ramirez</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>05:46:59 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Juan Emilio Perez Ramirez</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>05:52:53 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Juan Emilio Perez Ramirez</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>06:11:15 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Juan Emilio Perez Ramirez</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>06:14:34 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Juan Emilio Perez Ramirez</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>06:15:20 PM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>